<commit_message>
update products and QGIS
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7188EF8B-540B-46DA-B0AA-885C6ACB39F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B63EFB-17F5-4D8C-B41F-B9BF71CE0CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="439">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -795,9 +795,6 @@
     <t>Recomendaciones al SINAE</t>
   </si>
   <si>
-    <t xml:space="preserve">Estar atentos a los próximos eventos de lluvia que se registren en la cuenca.   </t>
-  </si>
-  <si>
     <t xml:space="preserve">En las últimas horas se registraron precipitaciones de fuerte intensidad en la cuenca (promedio 62 mm) del río Cuareim. </t>
   </si>
   <si>
@@ -1278,12 +1275,6 @@
     <t>En los últimos días se registraron lluvias en la cuenca del río Tacuarembó Chico, las cuales estuvieron en el entorno de 60 a 70 mm. No se prevé condiciones hidrologicas adversas en el río Negro, aunque no se descarta incrementos de nivel en la subcuenca del río Tacuarembó y Tacuarembó Chico.</t>
   </si>
   <si>
-    <t>Menor a 4.0 metros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entre las 07 horas 26 mayo hasta 07 horas del 27 mayo se registraró alrededor de 10 mm en promedio en la cuenca del río Olimar. Algunos modelos de pronóstico indican la posibilidad de lluvia pero que si llegan a ocurrir, el nivel del río Olimar en Treinta y Tres estaria por debajo de los 4 metros sin generar inconvenientes. </t>
-  </si>
-  <si>
     <t>Entre 5.50 y 6.10 metros</t>
   </si>
   <si>
@@ -1293,48 +1284,9 @@
     <t xml:space="preserve">Se mantiene en ascenso el nivel del río Uruguay. CTM-Salto Grande reporta en su comunicado diario que el caudal medio diario evacuado variará entre12000 y 13500 m3/s y la cota máxima y minima en Salto variará entre 8.50 y 9.70 metros. En Paysandú, el nivel del río se mantiene en ascenso y se espera que el río pueda alcanzar los 5 metros, lo cual indica que estaria por debajo de su cota de seguridad (6 metros). En relación a los ríos Daymán y Arapey se encuentran en descenso, mientras que el río Queguay se mantiene en ascenso y en una cota de 5.36 metros. </t>
   </si>
   <si>
-    <t>08 Abril</t>
-  </si>
-  <si>
-    <t>09 y 10 abril</t>
-  </si>
-  <si>
-    <t>Entre 10 y 11 abril</t>
-  </si>
-  <si>
-    <t>Menor a 4.50 m</t>
-  </si>
-  <si>
-    <t>Menor a 4.00 m</t>
-  </si>
-  <si>
     <t>Menor a 8.5 m</t>
   </si>
   <si>
-    <t xml:space="preserve">El río Cuareim se encuentra en descenso </t>
-  </si>
-  <si>
-    <t>Menor a 2.50 m</t>
-  </si>
-  <si>
-    <t>Menor a 3.00 m</t>
-  </si>
-  <si>
-    <t>En las ultimas horas se han registrado incrementos de nivel del río Yí en las localidades de Sarandí del Yí y Polanco del Yí. En la ciudad de Durazno se observó un incremento del caudal del río, el cual permanece en un nivel entorno a los 0.85 m en Puente Viejo. Con este escenario actual se espera que siga el ascenso el nivel del río, sin embargo no se espera que alcance la cota de aviso los próximos días.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Durante las últimas horas se registró el nivel máximo del río Cuareim en Artigas el cual alcanzó los 6.14 metros, sin acercarse a la cota de aviso (8.00 m). Actualmente el nivel del río se encuentra en descenso y no se espera nuevo incrementos en los próximos días. </t>
-  </si>
-  <si>
-    <t>24000 y 30000</t>
-  </si>
-  <si>
-    <t>150 y 375</t>
-  </si>
-  <si>
-    <t>375 y 500</t>
-  </si>
-  <si>
     <t>Mantener la vigilancia y el monitoreo en niveles de ríos y arroyos. Infórmese por fuentes oficiales</t>
   </si>
   <si>
@@ -1345,6 +1297,69 @@
   </si>
   <si>
     <t>Tomar acción en realizar evacuaciones debido a la posibilidad de generarse inundaciones que afecten viviendas, infraestructura sensible y equipamientos urbanos</t>
+  </si>
+  <si>
+    <t>6000 y 7700</t>
+  </si>
+  <si>
+    <t>132 y 289</t>
+  </si>
+  <si>
+    <t>265 y 462</t>
+  </si>
+  <si>
+    <t>Se registran incrementos de nivel en los ríos que transitan en zona centro, este, noreste y litoral norte del pais</t>
+  </si>
+  <si>
+    <t>En los ultimos días se registraron precipitaciones en el orden de los 90mm en la cuenca del río Yi. El nivel del río se encuentra en ascenso en las localidades de Sarandí del Yí, Polanco del Yí y en la ciudad de Durazno. Se espera que el nivel del río siga en ascenso en la ciudad de Durazno y sobrepase la cota de aviso (6.05m en puente viejo) generando inundaciones en la zona de camping. Con base en el pronóstico de precipitación actual no se espera que el nivel del río sobrepase la cota de seguridad, por lo tanto, no se esperan afectaciones a viviendas.</t>
+  </si>
+  <si>
+    <t>En el día de ayer se registraron precipitaciones en la cuenca del río Cuareím en el orden de los 50mm. El nivel del río se encuentra en ascenso en Catalán Grande y Cuareím Río. Considerando los pronósticos de precipitación actuales, se espera que el nivel del río se mantenga en ascenso en la ciudad de Artigas y con posibilidad de aproximación a la cota de aviso (8.00 m). Así mismo, no se esperan inundaciones importantes en la zona del paseo 7 de Septiembre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En los últimos días se registraron precipitaciones abundantes en la cuenca del río Olimar, superando los 100mm en promedio. Considerando que no se esperan precipitaciones significativas en la cuenca en los próximos días, se espera que se mantenga el nivel del río en ascenso con posibilidad de registran un nivel máximo entre 5.70 a 6.70 metros entre el 21 y 22 de Julio. Este nivel pronosticado es cercano a la cota de seguridad (7.0 m) y no se descarta la posibilidad de aproximación. </t>
+  </si>
+  <si>
+    <t>Estar atentos a inundaciones en los primeros equipamientos colectivos expuesto de la localidad por la crecida. No descartar aún la posibilidad de afectación a las primeras viviendas de uso permanete en la trama urbana.</t>
+  </si>
+  <si>
+    <t>Menor a 7.00 m</t>
+  </si>
+  <si>
+    <t>Entre 20 y 21 julio</t>
+  </si>
+  <si>
+    <t>Menor a 10.00 m</t>
+  </si>
+  <si>
+    <t>21 de julio</t>
+  </si>
+  <si>
+    <t>Menor a 8.00 m</t>
+  </si>
+  <si>
+    <t>Menor a 9.00 m</t>
+  </si>
+  <si>
+    <t>Entre 22 y 23 julio</t>
+  </si>
+  <si>
+    <t>20 de julio</t>
+  </si>
+  <si>
+    <t>Menor a 7.5 m</t>
+  </si>
+  <si>
+    <t>Menor a 8.0 m</t>
+  </si>
+  <si>
+    <t>Entre 21 y 22 julio</t>
+  </si>
+  <si>
+    <t>Entre 5.70 a 6.70 metros</t>
+  </si>
+  <si>
+    <t>Entre 21 y 22 de julio</t>
   </si>
 </sst>
 </file>
@@ -2208,7 +2223,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="39">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2220,7 +2235,7 @@
       </c>
       <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46163</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2232,7 +2247,7 @@
       </c>
       <c r="C4" s="41">
         <f ca="1">$C$3-1</f>
-        <v>46162</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2244,7 +2259,7 @@
       </c>
       <c r="C5" s="40">
         <f ca="1">$C$3-2</f>
-        <v>46161</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2256,7 +2271,7 @@
       </c>
       <c r="C6" s="41">
         <f ca="1">$C$3+1</f>
-        <v>46164</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2268,7 +2283,7 @@
       </c>
       <c r="C7" s="42">
         <f ca="1">$C$3+2</f>
-        <v>46165</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2280,7 +2295,7 @@
       </c>
       <c r="C8" s="40">
         <f ca="1">$C$3+3</f>
-        <v>46166</v>
+        <v>46225</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2291,7 +2306,7 @@
         <v>171</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -2312,16 +2327,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
+        <v>339</v>
+      </c>
+      <c r="B1" s="57" t="s">
         <v>340</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="C1" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="C1" s="60" t="s">
-        <v>342</v>
-      </c>
       <c r="D1" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2329,13 +2344,13 @@
         <v>45224</v>
       </c>
       <c r="B2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C2" s="61" t="s">
         <v>343</v>
       </c>
-      <c r="C2" s="61" t="s">
-        <v>344</v>
-      </c>
       <c r="D2" s="61" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2343,10 +2358,10 @@
         <v>45224</v>
       </c>
       <c r="B3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C3" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2354,13 +2369,13 @@
         <v>45224</v>
       </c>
       <c r="B4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2368,10 +2383,10 @@
         <v>45224</v>
       </c>
       <c r="B5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C5" s="61" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2379,10 +2394,10 @@
         <v>45224</v>
       </c>
       <c r="B6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D6" s="62" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2390,13 +2405,13 @@
         <v>45224</v>
       </c>
       <c r="B7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C7" s="61" t="s">
+        <v>357</v>
+      </c>
+      <c r="D7" s="61" t="s">
         <v>358</v>
-      </c>
-      <c r="D7" s="61" t="s">
-        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -2435,7 +2450,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="72">
-        <v>1.56</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2446,7 +2461,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="71">
-        <v>1.78</v>
+        <v>5.96</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2456,9 +2471,9 @@
       <c r="B4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="30" t="str">
+      <c r="C4" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2470,7 +2485,7 @@
       </c>
       <c r="C5" s="37" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2481,7 +2496,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="72">
-        <v>2.4300000000000002</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2492,15 +2507,15 @@
         <v>7</v>
       </c>
       <c r="C7" s="71">
-        <v>2.44</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>336</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>337</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>248</v>
@@ -2513,9 +2528,9 @@
       <c r="B9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="30" t="str">
+      <c r="C9" s="30">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v/>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2527,7 +2542,7 @@
       </c>
       <c r="C10" s="37" t="str">
         <f>IF(C9=0,"Permanece",IF(C9="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2538,7 +2553,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="72">
-        <v>0.73</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2549,15 +2564,15 @@
         <v>11</v>
       </c>
       <c r="C12" s="71">
-        <v>0.73</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C13" s="6"/>
     </row>
@@ -2570,7 +2585,7 @@
       </c>
       <c r="C14" s="30">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2582,7 +2597,7 @@
       </c>
       <c r="C15" s="37" t="str">
         <f>IF(C14=0,"Permanece",IF(C14="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2593,7 +2608,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="71">
-        <v>2.2999999999999998</v>
+        <v>3.04</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2604,15 +2619,15 @@
         <v>14</v>
       </c>
       <c r="C17" s="71">
-        <v>2.2999999999999998</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C18" s="6"/>
     </row>
@@ -2625,7 +2640,7 @@
       </c>
       <c r="C19" s="30">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2637,7 +2652,7 @@
       </c>
       <c r="C20" s="37" t="str">
         <f>IF(C19=0,"Permanece",IF(C19="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2648,7 +2663,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="74">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2659,7 +2674,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="75">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2670,7 +2685,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="75">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2681,7 +2696,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="75">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2692,7 +2707,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2714,7 +2729,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2725,18 +2740,18 @@
         <v>35</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2747,7 +2762,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>418</v>
+        <v>429</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2758,7 +2773,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2769,7 +2784,7 @@
         <v>37</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>418</v>
+        <v>432</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2780,7 +2795,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>419</v>
+        <v>431</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2791,10 +2806,10 @@
         <v>38</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="198.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="26" t="s">
         <v>64</v>
       </c>
@@ -2802,7 +2817,7 @@
         <v>39</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2813,7 +2828,7 @@
         <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -2870,7 +2885,7 @@
         <v>82</v>
       </c>
       <c r="C2" s="71">
-        <v>3.93</v>
+        <v>4.3099999999999996</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2881,15 +2896,15 @@
         <v>83</v>
       </c>
       <c r="C3" s="71">
-        <v>3.92</v>
+        <v>4.2300000000000004</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>330</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>331</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -2904,7 +2919,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2927,7 +2942,7 @@
         <v>88</v>
       </c>
       <c r="C7" s="71">
-        <v>0.34</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2938,15 +2953,15 @@
         <v>89</v>
       </c>
       <c r="C8" s="71">
-        <v>0.34</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
+        <v>331</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>332</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>333</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>248</v>
@@ -2961,7 +2976,7 @@
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2973,7 +2988,7 @@
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2984,7 +2999,7 @@
         <v>94</v>
       </c>
       <c r="C12" s="71">
-        <v>1.83</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2995,15 +3010,15 @@
         <v>95</v>
       </c>
       <c r="C13" s="71">
-        <v>1.83</v>
+        <v>2.5099999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>248</v>
@@ -3018,7 +3033,7 @@
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3030,7 +3045,7 @@
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -3041,7 +3056,7 @@
         <v>74</v>
       </c>
       <c r="C17" s="74">
-        <v>0</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3052,7 +3067,7 @@
         <v>75</v>
       </c>
       <c r="C18" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -3074,7 +3089,7 @@
         <v>77</v>
       </c>
       <c r="C20" s="75">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3085,7 +3100,7 @@
         <v>78</v>
       </c>
       <c r="C21" s="75">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3107,7 +3122,7 @@
         <v>86</v>
       </c>
       <c r="C23" s="73" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3118,7 +3133,7 @@
         <v>87</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>398</v>
+        <v>433</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3129,7 +3144,7 @@
         <v>92</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>398</v>
+        <v>434</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3140,7 +3155,7 @@
         <v>93</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>398</v>
+        <v>433</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -3151,7 +3166,7 @@
         <v>98</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>421</v>
+        <v>435</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3162,10 +3177,10 @@
         <v>99</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
         <v>64</v>
       </c>
@@ -3173,7 +3188,7 @@
         <v>80</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3184,7 +3199,7 @@
         <v>81</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>250</v>
+        <v>414</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3279,7 +3294,7 @@
         <v>162</v>
       </c>
       <c r="C2" s="72">
-        <v>0.55000000000000004</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3290,15 +3305,15 @@
         <v>163</v>
       </c>
       <c r="C3" s="71">
-        <v>0.55000000000000004</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>320</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>321</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -3313,7 +3328,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3325,7 +3340,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3348,10 +3363,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>322</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>323</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>248</v>
@@ -3389,7 +3404,7 @@
         <v>166</v>
       </c>
       <c r="C12" s="72">
-        <v>1.48</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3400,15 +3415,15 @@
         <v>167</v>
       </c>
       <c r="C13" s="71">
-        <v>1.48</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
+        <v>325</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>326</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>327</v>
       </c>
       <c r="C14" s="6"/>
     </row>
@@ -3456,10 +3471,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>328</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>329</v>
       </c>
       <c r="C19" s="6"/>
     </row>
@@ -3495,7 +3510,7 @@
         <v>112</v>
       </c>
       <c r="C22" s="74">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -3506,7 +3521,7 @@
         <v>113</v>
       </c>
       <c r="C23" s="75">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3517,7 +3532,7 @@
         <v>114</v>
       </c>
       <c r="C24" s="76">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3528,7 +3543,7 @@
         <v>115</v>
       </c>
       <c r="C25" s="75">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3539,7 +3554,7 @@
         <v>116</v>
       </c>
       <c r="C26" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3555,24 +3570,24 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3583,7 +3598,7 @@
         <v>120</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3594,7 +3609,7 @@
         <v>121</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -3605,7 +3620,7 @@
         <v>126</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3616,24 +3631,24 @@
         <v>127</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C34" s="9"/>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C35" s="10"/>
     </row>
@@ -3645,7 +3660,7 @@
         <v>128</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3656,7 +3671,7 @@
         <v>129</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3667,7 +3682,7 @@
         <v>134</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3678,7 +3693,7 @@
         <v>135</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3689,7 +3704,7 @@
         <v>118</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3700,7 +3715,7 @@
         <v>119</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -3756,7 +3771,7 @@
         <v>154</v>
       </c>
       <c r="C2" s="72">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3767,15 +3782,15 @@
         <v>155</v>
       </c>
       <c r="C3" s="72">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -3810,10 +3825,10 @@
         <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C7" s="74">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3821,10 +3836,10 @@
         <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C8" s="75">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3832,7 +3847,7 @@
         <v>53</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C9" s="76">
         <v>0</v>
@@ -3843,10 +3858,10 @@
         <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C10" s="75">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3854,10 +3869,10 @@
         <v>56</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C11" s="75">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3865,7 +3880,7 @@
         <v>55</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C12" s="76">
         <v>0</v>
@@ -3879,7 +3894,7 @@
         <v>160</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3890,7 +3905,7 @@
         <v>161</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3898,10 +3913,10 @@
         <v>64</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3909,10 +3924,10 @@
         <v>65</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -3969,7 +3984,7 @@
         <v>205</v>
       </c>
       <c r="C2" s="72">
-        <v>2.36</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3980,15 +3995,15 @@
         <v>206</v>
       </c>
       <c r="C3" s="71">
-        <v>2.36</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>309</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -4027,7 +4042,7 @@
         <v>209</v>
       </c>
       <c r="C7" s="72">
-        <v>2.21</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4038,15 +4053,15 @@
         <v>210</v>
       </c>
       <c r="C8" s="71">
-        <v>2.21</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>310</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>311</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>248</v>
@@ -4061,7 +4076,7 @@
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" s="55"/>
     </row>
@@ -4074,7 +4089,7 @@
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -4085,7 +4100,7 @@
         <v>176</v>
       </c>
       <c r="C12" s="72">
-        <v>3.11</v>
+        <v>5.74</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -4096,15 +4111,15 @@
         <v>177</v>
       </c>
       <c r="C13" s="71">
-        <v>2.96</v>
+        <v>5.76</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>312</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>313</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>248</v>
@@ -4117,9 +4132,9 @@
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="C15" s="30">
+      <c r="C15" s="30" t="str">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>15</v>
+        <v/>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4131,7 +4146,7 @@
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4142,7 +4157,7 @@
         <v>213</v>
       </c>
       <c r="C17" s="72">
-        <v>1.37</v>
+        <v>2.4700000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -4153,18 +4168,18 @@
         <v>214</v>
       </c>
       <c r="C18" s="71">
-        <v>1.37</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>315</v>
-      </c>
       <c r="C19" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -4176,7 +4191,7 @@
       </c>
       <c r="C20" s="30">
         <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4188,7 +4203,7 @@
       </c>
       <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -4199,7 +4214,7 @@
         <v>217</v>
       </c>
       <c r="C22" s="72">
-        <v>1.51</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -4210,15 +4225,15 @@
         <v>218</v>
       </c>
       <c r="C23" s="71">
-        <v>1.52</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
+        <v>315</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>316</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>317</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>248</v>
@@ -4258,7 +4273,7 @@
         <v>174</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -4269,7 +4284,7 @@
         <v>172</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4307,7 +4322,7 @@
         <v>199</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4345,7 +4360,7 @@
         <v>196</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4356,7 +4371,7 @@
         <v>221</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -4412,7 +4427,7 @@
         <v>224</v>
       </c>
       <c r="C2" s="72">
-        <v>9.56</v>
+        <v>6.91</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4423,15 +4438,15 @@
         <v>225</v>
       </c>
       <c r="C3" s="71">
-        <v>9.56</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>318</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>319</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -4446,7 +4461,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4458,7 +4473,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4469,7 +4484,7 @@
         <v>230</v>
       </c>
       <c r="C7" s="72">
-        <v>1.91</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4480,15 +4495,15 @@
         <v>231</v>
       </c>
       <c r="C8" s="71">
-        <v>1.92</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>248</v>
@@ -4501,9 +4516,9 @@
       <c r="B10" s="29" t="s">
         <v>232</v>
       </c>
-      <c r="C10" s="30" t="str">
+      <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4515,7 +4530,7 @@
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -4526,7 +4541,7 @@
         <v>237</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4537,7 +4552,7 @@
         <v>236</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4584,7 +4599,7 @@
         <v>246</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4595,7 +4610,7 @@
         <v>247</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -4645,32 +4660,32 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C2" s="72">
-        <v>0.35</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C3" s="71">
-        <v>0.36</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>248</v>
@@ -4681,11 +4696,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>370</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>369</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4693,11 +4708,11 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4705,10 +4720,10 @@
         <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C7" s="74">
-        <v>0</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4716,10 +4731,10 @@
         <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C8" s="75">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4727,10 +4742,10 @@
         <v>53</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C9" s="75">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4738,10 +4753,10 @@
         <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C10" s="75">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4749,10 +4764,10 @@
         <v>56</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C11" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4760,7 +4775,7 @@
         <v>55</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C12" s="76">
         <v>0</v>
@@ -4768,44 +4783,46 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>411</v>
+        <v>437</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>378</v>
-      </c>
-      <c r="C14" s="10"/>
-    </row>
-    <row r="15" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>377</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
         <v>64</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="28" t="s">
         <v>65</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -4856,7 +4873,7 @@
         <v>249</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D1" s="49"/>
       <c r="E1" s="49"/>
@@ -4871,29 +4888,29 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>430</v>
+        <v>414</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D2" s="47" t="s">
+        <v>260</v>
+      </c>
+      <c r="E2" s="47" t="s">
         <v>261</v>
       </c>
-      <c r="E2" s="47" t="s">
-        <v>262</v>
-      </c>
       <c r="F2" s="48" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G2" s="54"/>
       <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="s">
-        <v>431</v>
+        <v>415</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D3" s="45">
         <v>70</v>
@@ -4902,24 +4919,24 @@
         <v>200</v>
       </c>
       <c r="F3" s="45" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I3" s="45" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J3" s="45" t="s">
+        <v>254</v>
+      </c>
+      <c r="K3" s="45" t="s">
         <v>255</v>
-      </c>
-      <c r="K3" s="45" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
-        <v>432</v>
+        <v>416</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D4" s="45">
         <v>30</v>
@@ -4928,23 +4945,23 @@
         <v>100</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="45" t="s">
-        <v>433</v>
+        <v>417</v>
       </c>
       <c r="F5" s="45" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E7" s="47" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G7" s="46"/>
       <c r="H7" s="46"/>
@@ -4956,49 +4973,49 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E8" s="45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F8" s="45" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I8" s="45" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J8" s="45" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E9" s="45" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E10" s="45" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I10" s="45" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C12" s="47" t="s">
+        <v>265</v>
+      </c>
+      <c r="D12" s="47" t="s">
+        <v>263</v>
+      </c>
+      <c r="E12" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="D12" s="47" t="s">
-        <v>264</v>
-      </c>
-      <c r="E12" s="47" t="s">
-        <v>267</v>
-      </c>
       <c r="F12" s="46" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G12" s="46"/>
       <c r="H12" s="46"/>
@@ -5010,43 +5027,43 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D13" s="45" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F13" s="45" t="s">
+        <v>351</v>
+      </c>
+      <c r="I13" s="45" t="s">
         <v>352</v>
-      </c>
-      <c r="I13" s="45" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D14" s="45" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I14" s="45" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D15" s="45" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I15" s="45" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="47" t="s">
+        <v>265</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>263</v>
+      </c>
+      <c r="E17" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="D17" s="47" t="s">
-        <v>264</v>
-      </c>
-      <c r="E17" s="47" t="s">
-        <v>267</v>
-      </c>
       <c r="F17" s="46" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G17" s="46"/>
       <c r="H17" s="46"/>
@@ -5058,67 +5075,67 @@
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F18" s="45" t="s">
+        <v>256</v>
+      </c>
+      <c r="I18" s="45" t="s">
         <v>257</v>
-      </c>
-      <c r="I18" s="45" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F19" s="45" t="s">
+        <v>258</v>
+      </c>
+      <c r="I19" s="45" t="s">
         <v>259</v>
-      </c>
-      <c r="I19" s="45" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="50" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E22" s="50" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F22" s="50" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G22" s="50"/>
       <c r="H22" s="50"/>
       <c r="I22" s="50" t="s">
+        <v>294</v>
+      </c>
+      <c r="J22" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="J22" s="50" t="s">
+      <c r="K22" s="50" t="s">
         <v>296</v>
       </c>
-      <c r="K22" s="50" t="s">
-        <v>297</v>
-      </c>
       <c r="L22" s="69" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="23" spans="3:13" s="63" customFormat="1" ht="99" x14ac:dyDescent="0.25">
       <c r="C23" s="63" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E23" s="63" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 56 mm/día.</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
       <c r="I23" s="52" t="str">
         <f>_xlfn.CONCAT($F$8,D23,IF(YI!C15=$E$8,$I$8,IF(YI!C15=$E$9,$I$9,$I$10)),$J$8,E23,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno. </v>
       </c>
       <c r="J23" s="52" t="str">
         <f>_xlfn.CONCAT(F13,IF(YI!C31&gt;YI!C11,I13, IF(YI!C31=YI!C11,I14, I15)))</f>
@@ -5130,28 +5147,28 @@
       </c>
       <c r="L23" s="52" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 56 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
       <c r="C24" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="D24" s="51" t="s">
         <v>284</v>
       </c>
-      <c r="D24" s="51" t="s">
-        <v>285</v>
-      </c>
       <c r="E24" s="51" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 54 mm y con un máximo de 53 mm/día.</v>
       </c>
       <c r="G24" s="53"/>
       <c r="H24" s="53"/>
       <c r="I24" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D24,IF(CUAREIM!C16=$E$8,$I$8,IF(CUAREIM!C16=$E$9,$I$9,$I$10)),$J$8,E24,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Cuareim se mantiene constante en la ciudad de Artigas. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas. </v>
       </c>
       <c r="J24" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(CUAREIM!C27&gt;CUAREIM!C12,I13, IF(CUAREIM!C27=CUAREIM!C12,I14, I15)))</f>
@@ -5163,22 +5180,22 @@
       </c>
       <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Cuareim se mantiene constante en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 54 mm y con un máximo de 53 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
       <c r="C25" s="51" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 29 mm/día.</v>
       </c>
       <c r="G25" s="52"/>
       <c r="H25" s="52"/>
@@ -5196,18 +5213,18 @@
       </c>
       <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 29 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="51" t="s">
+        <v>286</v>
+      </c>
+      <c r="D26" s="51" t="s">
         <v>287</v>
       </c>
-      <c r="D26" s="51" t="s">
+      <c r="E26" s="51" t="s">
         <v>288</v>
-      </c>
-      <c r="E26" s="51" t="s">
-        <v>289</v>
       </c>
       <c r="F26" s="77" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!#REF!)&gt;$D$3,SUM(URUGUAY!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!#REF!)&gt;$D$4,SUM(URUGUAY!#REF!)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!#REF!),$J$3,MAX(URUGUAY!#REF!),$K$3)</f>
@@ -5215,7 +5232,7 @@
       </c>
       <c r="I26" s="64" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en la ciudad de  Salto; se mantiene constante en las ciudades de Bella Unión Paysandú; está en descenso en la ciudad de  Fray Bentos.</v>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de ; está en descenso en las ciudades de Salto Fray Bentos.</v>
       </c>
       <c r="J26" s="78" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C28&gt;URUGUAY!C7, URUGUAY!C30&gt;URUGUAY!C12, URUGUAY!C32&gt;URUGUAY!C17, URUGUAY!C34&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C28=URUGUAY!C7, URUGUAY!C30=URUGUAY!C12, URUGUAY!C32=URUGUAY!C17, URUGUAY!C34=URUGUAY!C22),I14, I15)))</f>
@@ -5230,70 +5247,70 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="27" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
       <c r="C27" s="51"/>
       <c r="D27" s="51"/>
       <c r="E27" s="51" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F27" s="77"/>
       <c r="G27" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E8, URUGUAY!$C$16=Tablas!E8,URUGUAY!$C$21=Tablas!E8,URUGUAY!$C$26=Tablas!E8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H27" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E8,_xlfn.CONCAT(" ",$E$26,),""),IF(URUGUAY!$C$16=Tablas!E8,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E8,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E8,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto</v>
+        <v xml:space="preserve"> Bella Unión Paysandú</v>
       </c>
       <c r="I27" s="65" t="str">
         <f>_xlfn.CONCAT(I8,IF(G27&gt;1,$J$9,$J$8),H27, IF(G27=4,".", ";"))</f>
-        <v xml:space="preserve"> está en ascenso en la ciudad de  Salto;</v>
+        <v xml:space="preserve"> está en ascenso en las ciudades de Bella Unión Paysandú;</v>
       </c>
       <c r="J27" s="78"/>
       <c r="K27" s="78"/>
       <c r="L27" s="78"/>
     </row>
-    <row r="28" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="51"/>
       <c r="D28" s="51"/>
       <c r="E28" s="51" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F28" s="77"/>
       <c r="G28" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H28" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Bella Unión Paysandú</v>
+        <v/>
       </c>
       <c r="I28" s="65" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en las ciudades de Bella Unión Paysandú;</v>
+        <v xml:space="preserve"> se mantiene constante en la ciudad de ;</v>
       </c>
       <c r="J28" s="78"/>
       <c r="K28" s="78"/>
       <c r="L28" s="78"/>
     </row>
-    <row r="29" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:13" ht="33" x14ac:dyDescent="0.3">
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
       <c r="E29" s="51" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F29" s="77"/>
       <c r="G29" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Fray Bentos</v>
+        <v xml:space="preserve"> Salto Fray Bentos</v>
       </c>
       <c r="I29" s="65" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
-        <v xml:space="preserve"> está en descenso en la ciudad de  Fray Bentos.</v>
+        <v xml:space="preserve"> está en descenso en las ciudades de Salto Fray Bentos.</v>
       </c>
       <c r="J29" s="78"/>
       <c r="K29" s="78"/>
@@ -5301,13 +5318,13 @@
     </row>
     <row r="30" spans="3:13" ht="66" x14ac:dyDescent="0.3">
       <c r="C30" s="51" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D30" s="51" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E30" s="51" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F30" s="52" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!#REF!)&gt;$D$3,SUM(NEGRO!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!#REF!)&gt;$D$4,SUM(NEGRO!#REF!)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!#REF!),$J$3,MAX(NEGRO!#REF!),$K$3)</f>
@@ -5317,7 +5334,7 @@
       <c r="H30" s="52"/>
       <c r="I30" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D30,IF(NEGRO!C11=$E$8,$I$8,IF(NEGRO!C11=$E$9,$I$9,$I$10)),$J$8,E30,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en descenso en la ciudad de Mercedes. </v>
+        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en ascenso en la ciudad de Mercedes. </v>
       </c>
       <c r="J30" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(NEGRO!C16&gt;NEGRO!C7,I13, IF(NEGRO!C16=NEGRO!C7,I14, I15)))</f>

</xml_diff>

<commit_message>
new update of the doc master and qgis
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B63EFB-17F5-4D8C-B41F-B9BF71CE0CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEB8EF4-0734-4B2F-9164-A01C45A177D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="433">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -1239,12 +1239,6 @@
     <t xml:space="preserve"> -</t>
   </si>
   <si>
-    <t>29/05</t>
-  </si>
-  <si>
-    <t>Estar atentos a los pronósticos meteorológicos que realiza el INUMET y a la red pluviométrica y de medición de nivel del río Santa Lucía.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Estar atentos a los pronósticos meteorológicos que realiza el INUMET y a los próximos eventos de lluvia que se registren en la cuenca. </t>
   </si>
   <si>
@@ -1254,39 +1248,9 @@
     <t>Menor a 5 metros</t>
   </si>
   <si>
-    <t>29 mayo</t>
-  </si>
-  <si>
-    <t>30 mayo</t>
-  </si>
-  <si>
     <t>Menor a 3 metros</t>
   </si>
   <si>
-    <t xml:space="preserve">Entre las 07 horas 26 mayo hasta las 07 horas del 27 mayo 2025, se registró precipitaciones en la cuenca del río Santa Lucia, las cuales fueron en el entorno de 10 mm en promedio. Algunos modelos meteorológico indican la posibilidad de precipitaciones en las próxima hora. Si este escenario sucede, se esperaria que el nivel del río aumente pero sin generar ningún inconveniente en la actividades cotidianas en las localidades dentro de la cuenca. </t>
-  </si>
-  <si>
-    <t>Menor a 3.2 metros</t>
-  </si>
-  <si>
-    <t>Entre las 07 horas 26 mayo hasta 07 horas 27 mayo 2025, las precipitaciones en la cuenca del río San José fueron cercana a los 14 mm. Se espera que el nivel del río aumente ligeramente pero sin generar inconvenientes en la ciudad de San José</t>
-  </si>
-  <si>
-    <t>En los últimos días se registraron lluvias en la cuenca del río Tacuarembó Chico, las cuales estuvieron en el entorno de 60 a 70 mm. No se prevé condiciones hidrologicas adversas en el río Negro, aunque no se descarta incrementos de nivel en la subcuenca del río Tacuarembó y Tacuarembó Chico.</t>
-  </si>
-  <si>
-    <t>Entre 5.50 y 6.10 metros</t>
-  </si>
-  <si>
-    <t>Entre 4.50 y 5.00 metros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se mantiene en ascenso el nivel del río Uruguay. CTM-Salto Grande reporta en su comunicado diario que el caudal medio diario evacuado variará entre12000 y 13500 m3/s y la cota máxima y minima en Salto variará entre 8.50 y 9.70 metros. En Paysandú, el nivel del río se mantiene en ascenso y se espera que el río pueda alcanzar los 5 metros, lo cual indica que estaria por debajo de su cota de seguridad (6 metros). En relación a los ríos Daymán y Arapey se encuentran en descenso, mientras que el río Queguay se mantiene en ascenso y en una cota de 5.36 metros. </t>
-  </si>
-  <si>
-    <t>Menor a 8.5 m</t>
-  </si>
-  <si>
     <t>Mantener la vigilancia y el monitoreo en niveles de ríos y arroyos. Infórmese por fuentes oficiales</t>
   </si>
   <si>
@@ -1302,57 +1266,12 @@
     <t>6000 y 7700</t>
   </si>
   <si>
-    <t>132 y 289</t>
-  </si>
-  <si>
-    <t>265 y 462</t>
-  </si>
-  <si>
-    <t>Se registran incrementos de nivel en los ríos que transitan en zona centro, este, noreste y litoral norte del pais</t>
-  </si>
-  <si>
-    <t>En los ultimos días se registraron precipitaciones en el orden de los 90mm en la cuenca del río Yi. El nivel del río se encuentra en ascenso en las localidades de Sarandí del Yí, Polanco del Yí y en la ciudad de Durazno. Se espera que el nivel del río siga en ascenso en la ciudad de Durazno y sobrepase la cota de aviso (6.05m en puente viejo) generando inundaciones en la zona de camping. Con base en el pronóstico de precipitación actual no se espera que el nivel del río sobrepase la cota de seguridad, por lo tanto, no se esperan afectaciones a viviendas.</t>
-  </si>
-  <si>
-    <t>En el día de ayer se registraron precipitaciones en la cuenca del río Cuareím en el orden de los 50mm. El nivel del río se encuentra en ascenso en Catalán Grande y Cuareím Río. Considerando los pronósticos de precipitación actuales, se espera que el nivel del río se mantenga en ascenso en la ciudad de Artigas y con posibilidad de aproximación a la cota de aviso (8.00 m). Así mismo, no se esperan inundaciones importantes en la zona del paseo 7 de Septiembre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En los últimos días se registraron precipitaciones abundantes en la cuenca del río Olimar, superando los 100mm en promedio. Considerando que no se esperan precipitaciones significativas en la cuenca en los próximos días, se espera que se mantenga el nivel del río en ascenso con posibilidad de registran un nivel máximo entre 5.70 a 6.70 metros entre el 21 y 22 de Julio. Este nivel pronosticado es cercano a la cota de seguridad (7.0 m) y no se descarta la posibilidad de aproximación. </t>
-  </si>
-  <si>
-    <t>Estar atentos a inundaciones en los primeros equipamientos colectivos expuesto de la localidad por la crecida. No descartar aún la posibilidad de afectación a las primeras viviendas de uso permanete en la trama urbana.</t>
-  </si>
-  <si>
-    <t>Menor a 7.00 m</t>
-  </si>
-  <si>
     <t>Entre 20 y 21 julio</t>
   </si>
   <si>
-    <t>Menor a 10.00 m</t>
-  </si>
-  <si>
-    <t>21 de julio</t>
-  </si>
-  <si>
-    <t>Menor a 8.00 m</t>
-  </si>
-  <si>
     <t>Menor a 9.00 m</t>
   </si>
   <si>
-    <t>Entre 22 y 23 julio</t>
-  </si>
-  <si>
-    <t>20 de julio</t>
-  </si>
-  <si>
-    <t>Menor a 7.5 m</t>
-  </si>
-  <si>
-    <t>Menor a 8.0 m</t>
-  </si>
-  <si>
     <t>Entre 21 y 22 julio</t>
   </si>
   <si>
@@ -1360,6 +1279,69 @@
   </si>
   <si>
     <t>Entre 21 y 22 de julio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se mantiene incrementos de nivel en ríos y arroyos que transitan en la zona noreste, litoral norte, centro y este del país. </t>
+  </si>
+  <si>
+    <t>Entre 8.33 a 9.00 metros</t>
+  </si>
+  <si>
+    <t>Entre 8.40 a 9.00 metros</t>
+  </si>
+  <si>
+    <t>Entre 7.40 a 8.10 metros</t>
+  </si>
+  <si>
+    <t>Entre 23 y 24 julio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debido a las precipitaciones registradas en los últimos días, se mantiene el incremento del caudal del río Yí en los sitios Polanco del Yí y Durazno. El día de ayer se registró el nivel máximo en Sarandí del Yí que alcanzó los 7.50 metros como nivel máximo. En base a este escenario se espera que se mantenga en ascenso el nivel del río Yí y con posibilidades de superar la cota de aviso (6 metros) y alcanzar la cota de seguridad (8.20 metros) en la ciudad de Durazno Puente Viejo. Este nivel máximo se esperaría entre 23 y 24 de julio 2026 con posibilidad de generar impactos como cierre puente Capurro, inundación en zona de camping e inundaciones en la ciudad de Durazno y Santa Bernandina. </t>
+  </si>
+  <si>
+    <t>Se recomienda estar preparados antes afectaciones por inundaciones en Durazno y Santa Bernandina</t>
+  </si>
+  <si>
+    <t>Menor a 8.50 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se mantiene en ascenso el nivel del río Cuareim en Artigas, el cual se espera que pueda superar la cota de aviso (8.0 m) definido para la ciudad y alcanzar un nivel máximo inferior a los 9.00 metros. Este nivel representaria inundaciones en la zona del paseo 7 de setiembre y alrededores de estadio Matias Gonzalez en Artigas.  La posibilidad de alcanzar cota de seguridad (10.0 m) por el momento se mantiene baja. </t>
+  </si>
+  <si>
+    <t>22 julio</t>
+  </si>
+  <si>
+    <t>21 julio</t>
+  </si>
+  <si>
+    <t>Se registraron precipitaciones en la cuenca del río Santa Lucia y se observa incrementos de nivel que se mantiene por debajo de cota de aviso y seguridad para las diferentes localidades dentro de la cuenca</t>
+  </si>
+  <si>
+    <t>Menor a 2.0 metros</t>
+  </si>
+  <si>
+    <t>Se espera incrementos leves de nivel en el río San José los cuales estarian por debajo de la cota de seguridad</t>
+  </si>
+  <si>
+    <t>Entre 4.80 a 7.00 metros</t>
+  </si>
+  <si>
+    <t>Se mantiene en ascenso los niveles de los ríos Cuariem y Arapey debido a las precipitaciones registrada los días anteriores. De acuerdo a datos brindados por CTM-Salto Grande</t>
+  </si>
+  <si>
+    <t>163 y 487</t>
+  </si>
+  <si>
+    <t>265 y 872</t>
+  </si>
+  <si>
+    <t>En los últimos días se han registrados incrementos de nivel y caudal en los ríos Tacuarembó, Yí y el tramo del río Negro aguas arriba de la represa Rincón del Bonete. En la represa Hid. Constitución, UTE reporta que la previsión de erogados a erogar estaria entre 265 y 872 m3/s, sin embargo la previsión de niveles en Mercedes se mantendria por debajo de los 3.5 metros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En los últimos días se registraron precipitaciones abundantes en la cuenca del río Olimar, superando los 100mm en promedio. Considerando que no se esperan precipitaciones significativas en la cuenca en los próximos días, se espera que se mantenga el nivel del río en ascenso con posibilidad de registran un nivel máximo entre 6.00 a 6.80 metros entre el 21 y 22 de Julio. Este nivel pronosticado es cercano a la cota de seguridad (7.0 m) y no se descarta la posibilidad de aproximación. </t>
+  </si>
+  <si>
+    <t>Estar preparados a inundaciones en los primeros equipamientos colectivos expuesto de la localidad por la crecida. No descartar aún la posibilidad de afectación a las primeras viviendas de uso permanete en la trama urbana.</t>
   </si>
 </sst>
 </file>
@@ -2223,7 +2205,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2235,7 +2217,7 @@
       </c>
       <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46222</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2247,7 +2229,7 @@
       </c>
       <c r="C4" s="41">
         <f ca="1">$C$3-1</f>
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2259,7 +2241,7 @@
       </c>
       <c r="C5" s="40">
         <f ca="1">$C$3-2</f>
-        <v>46220</v>
+        <v>46221</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2271,7 +2253,7 @@
       </c>
       <c r="C6" s="41">
         <f ca="1">$C$3+1</f>
-        <v>46223</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2283,7 +2265,7 @@
       </c>
       <c r="C7" s="42">
         <f ca="1">$C$3+2</f>
-        <v>46224</v>
+        <v>46225</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2295,7 +2277,7 @@
       </c>
       <c r="C8" s="40">
         <f ca="1">$C$3+3</f>
-        <v>46225</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2306,7 +2288,7 @@
         <v>171</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
     </row>
   </sheetData>
@@ -2450,7 +2432,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="72">
-        <v>6.1</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2461,7 +2443,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="71">
-        <v>5.96</v>
+        <v>7.17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2471,9 +2453,9 @@
       <c r="B4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>14</v>
+        <v/>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2485,7 +2467,7 @@
       </c>
       <c r="C5" s="37" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2496,7 +2478,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="72">
-        <v>3.73</v>
+        <v>6.64</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2507,7 +2489,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="71">
-        <v>3.62</v>
+        <v>6.48</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2530,7 +2512,7 @@
       </c>
       <c r="C9" s="30">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2553,7 +2535,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="72">
-        <v>2.76</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2564,7 +2546,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="71">
-        <v>2.16</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2585,7 +2567,7 @@
       </c>
       <c r="C14" s="30">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
-        <v>60</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2608,7 +2590,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="71">
-        <v>3.04</v>
+        <v>6.19</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2619,7 +2601,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="71">
-        <v>2.91</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2640,7 +2622,7 @@
       </c>
       <c r="C19" s="30">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2663,7 +2645,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="74">
-        <v>56</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2674,7 +2656,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="75">
-        <v>23</v>
+        <v>67.400000000000006</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2685,7 +2667,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="75">
-        <v>9</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2696,7 +2678,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="75">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2707,7 +2689,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="75">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2729,7 +2711,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>426</v>
+        <v>248</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2740,7 +2722,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>427</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2751,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2762,7 +2744,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>429</v>
+        <v>409</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2773,7 +2755,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>430</v>
+        <v>414</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2784,7 +2766,7 @@
         <v>37</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>432</v>
+        <v>416</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2795,7 +2777,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>431</v>
+        <v>415</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2806,10 +2788,10 @@
         <v>38</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="198.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="264.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="26" t="s">
         <v>64</v>
       </c>
@@ -2817,10 +2799,10 @@
         <v>39</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="28" t="s">
         <v>65</v>
       </c>
@@ -2828,7 +2810,7 @@
         <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -2885,7 +2867,7 @@
         <v>82</v>
       </c>
       <c r="C2" s="71">
-        <v>4.3099999999999996</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2896,7 +2878,7 @@
         <v>83</v>
       </c>
       <c r="C3" s="71">
-        <v>4.2300000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2919,7 +2901,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2942,7 +2924,7 @@
         <v>88</v>
       </c>
       <c r="C7" s="71">
-        <v>0.98</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2953,7 +2935,7 @@
         <v>89</v>
       </c>
       <c r="C8" s="71">
-        <v>0.63</v>
+        <v>7.51</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2976,7 +2958,7 @@
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2999,7 +2981,7 @@
         <v>94</v>
       </c>
       <c r="C12" s="71">
-        <v>2.79</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3010,7 +2992,7 @@
         <v>95</v>
       </c>
       <c r="C13" s="71">
-        <v>2.5099999999999998</v>
+        <v>7.21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3033,7 +3015,7 @@
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>28</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3056,7 +3038,7 @@
         <v>74</v>
       </c>
       <c r="C17" s="74">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3067,7 +3049,7 @@
         <v>75</v>
       </c>
       <c r="C18" s="75">
-        <v>1</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -3089,7 +3071,7 @@
         <v>77</v>
       </c>
       <c r="C20" s="75">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3121,9 +3103,7 @@
       <c r="B23" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="73" t="s">
-        <v>413</v>
-      </c>
+      <c r="C23" s="73"/>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
@@ -3132,9 +3112,7 @@
       <c r="B24" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>433</v>
-      </c>
+      <c r="C24" s="9"/>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="26" t="s">
@@ -3144,7 +3122,7 @@
         <v>92</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>434</v>
+        <v>419</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3155,7 +3133,7 @@
         <v>93</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>433</v>
+        <v>407</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -3166,7 +3144,7 @@
         <v>98</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3177,10 +3155,10 @@
         <v>99</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
         <v>64</v>
       </c>
@@ -3188,10 +3166,10 @@
         <v>80</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="28" t="s">
         <v>65</v>
       </c>
@@ -3199,7 +3177,7 @@
         <v>81</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3294,7 +3272,7 @@
         <v>162</v>
       </c>
       <c r="C2" s="72">
-        <v>0.5</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3305,7 +3283,7 @@
         <v>163</v>
       </c>
       <c r="C3" s="71">
-        <v>0.48</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3404,7 +3382,7 @@
         <v>166</v>
       </c>
       <c r="C12" s="72">
-        <v>1.2</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3415,7 +3393,7 @@
         <v>167</v>
       </c>
       <c r="C13" s="71">
-        <v>1.2</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3436,7 +3414,7 @@
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3448,7 +3426,7 @@
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3510,7 +3488,7 @@
         <v>112</v>
       </c>
       <c r="C22" s="74">
-        <v>29</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -3521,7 +3499,7 @@
         <v>113</v>
       </c>
       <c r="C23" s="75">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3532,7 +3510,7 @@
         <v>114</v>
       </c>
       <c r="C24" s="76">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3543,7 +3521,7 @@
         <v>115</v>
       </c>
       <c r="C25" s="75">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3554,7 +3532,7 @@
         <v>116</v>
       </c>
       <c r="C26" s="75">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3576,7 +3554,7 @@
         <v>383</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3587,7 +3565,7 @@
         <v>384</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3598,7 +3576,7 @@
         <v>120</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3609,7 +3587,7 @@
         <v>121</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>403</v>
+        <v>422</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -3620,7 +3598,7 @@
         <v>126</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3631,7 +3609,7 @@
         <v>127</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>404</v>
+        <v>421</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -3641,7 +3619,9 @@
       <c r="B34" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="C34" s="9"/>
+      <c r="C34" s="9" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25" t="s">
@@ -3650,7 +3630,9 @@
       <c r="B35" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="C35" s="10"/>
+      <c r="C35" s="10" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="26" t="s">
@@ -3660,7 +3642,7 @@
         <v>128</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3671,7 +3653,7 @@
         <v>129</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>404</v>
+        <v>421</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3682,7 +3664,7 @@
         <v>134</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3693,10 +3675,10 @@
         <v>135</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="26" t="s">
         <v>64</v>
       </c>
@@ -3704,10 +3686,10 @@
         <v>118</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="28" t="s">
         <v>65</v>
       </c>
@@ -3715,7 +3697,7 @@
         <v>119</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -3828,7 +3810,7 @@
         <v>389</v>
       </c>
       <c r="C7" s="74">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3839,7 +3821,7 @@
         <v>390</v>
       </c>
       <c r="C8" s="75">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3850,7 +3832,7 @@
         <v>391</v>
       </c>
       <c r="C9" s="76">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3861,7 +3843,7 @@
         <v>392</v>
       </c>
       <c r="C10" s="75">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3872,7 +3854,7 @@
         <v>393</v>
       </c>
       <c r="C11" s="75">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3894,7 +3876,7 @@
         <v>160</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>407</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3905,10 +3887,10 @@
         <v>161</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
         <v>64</v>
       </c>
@@ -3916,7 +3898,7 @@
         <v>395</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>408</v>
+        <v>425</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3934,7 +3916,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{CB07A3A1-E957-443D-BA3B-C8739971E1B2}">
           <x14:formula1>
             <xm:f>Tablas!$L$25</xm:f>
@@ -3984,7 +3966,7 @@
         <v>205</v>
       </c>
       <c r="C2" s="72">
-        <v>4.51</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3995,7 +3977,7 @@
         <v>206</v>
       </c>
       <c r="C3" s="71">
-        <v>4.51</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -4016,9 +3998,9 @@
       <c r="B5" s="29" t="s">
         <v>207</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="D5" s="55"/>
     </row>
@@ -4031,7 +4013,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -4042,7 +4024,7 @@
         <v>209</v>
       </c>
       <c r="C7" s="72">
-        <v>3.46</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4053,7 +4035,7 @@
         <v>210</v>
       </c>
       <c r="C8" s="71">
-        <v>3.44</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4076,7 +4058,7 @@
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="55"/>
     </row>
@@ -4100,7 +4082,7 @@
         <v>176</v>
       </c>
       <c r="C12" s="72">
-        <v>5.74</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -4111,7 +4093,7 @@
         <v>177</v>
       </c>
       <c r="C13" s="71">
-        <v>5.76</v>
+        <v>6.48</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -4132,9 +4114,9 @@
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="C15" s="30" t="str">
+      <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v/>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4146,7 +4128,7 @@
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4157,7 +4139,7 @@
         <v>213</v>
       </c>
       <c r="C17" s="72">
-        <v>2.4700000000000002</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -4168,7 +4150,7 @@
         <v>214</v>
       </c>
       <c r="C18" s="71">
-        <v>2.42</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -4191,7 +4173,7 @@
       </c>
       <c r="C20" s="30">
         <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4203,7 +4185,7 @@
       </c>
       <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -4214,7 +4196,7 @@
         <v>217</v>
       </c>
       <c r="C22" s="72">
-        <v>1.67</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -4225,7 +4207,7 @@
         <v>218</v>
       </c>
       <c r="C23" s="71">
-        <v>1.69</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -4273,7 +4255,7 @@
         <v>174</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -4284,7 +4266,7 @@
         <v>172</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>410</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4294,7 +4276,9 @@
       <c r="B29" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C29" s="10"/>
+      <c r="C29" s="10" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
@@ -4303,7 +4287,9 @@
       <c r="B30" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C30" s="9"/>
+      <c r="C30" s="9" t="s">
+        <v>426</v>
+      </c>
     </row>
     <row r="31" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
@@ -4322,7 +4308,7 @@
         <v>199</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>411</v>
+        <v>248</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4332,7 +4318,9 @@
       <c r="B33" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="C33" s="10"/>
+      <c r="C33" s="10" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
@@ -4341,7 +4329,9 @@
       <c r="B34" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="C34" s="9"/>
+      <c r="C34" s="9" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27" t="s">
@@ -4350,9 +4340,11 @@
       <c r="B35" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C35" s="10"/>
-    </row>
-    <row r="36" spans="1:3" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C35" s="10" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="26" t="s">
         <v>64</v>
       </c>
@@ -4360,7 +4352,7 @@
         <v>196</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>412</v>
+        <v>427</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4371,7 +4363,7 @@
         <v>221</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -4427,7 +4419,7 @@
         <v>224</v>
       </c>
       <c r="C2" s="72">
-        <v>6.91</v>
+        <v>7.17</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4438,7 +4430,7 @@
         <v>225</v>
       </c>
       <c r="C3" s="71">
-        <v>6.88</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4459,9 +4451,9 @@
       <c r="B5" s="29" t="s">
         <v>226</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>3</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4473,7 +4465,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4484,7 +4476,7 @@
         <v>230</v>
       </c>
       <c r="C7" s="72">
-        <v>1.65</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4495,7 +4487,7 @@
         <v>231</v>
       </c>
       <c r="C8" s="71">
-        <v>1.63</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4518,7 +4510,7 @@
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4541,7 +4533,7 @@
         <v>237</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4552,7 +4544,7 @@
         <v>236</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4591,7 +4583,7 @@
       </c>
       <c r="C17" s="10"/>
     </row>
-    <row r="18" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
         <v>64</v>
       </c>
@@ -4599,7 +4591,7 @@
         <v>246</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>409</v>
+        <v>430</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4666,7 +4658,7 @@
         <v>366</v>
       </c>
       <c r="C2" s="72">
-        <v>-0.1</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4677,7 +4669,7 @@
         <v>367</v>
       </c>
       <c r="C3" s="71">
-        <v>-0.1</v>
+        <v>4.3099999999999996</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4700,7 +4692,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4712,7 +4704,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4723,7 +4715,7 @@
         <v>371</v>
       </c>
       <c r="C7" s="74">
-        <v>92</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4734,7 +4726,7 @@
         <v>372</v>
       </c>
       <c r="C8" s="75">
-        <v>25</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4745,7 +4737,7 @@
         <v>373</v>
       </c>
       <c r="C9" s="75">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4756,7 +4748,7 @@
         <v>374</v>
       </c>
       <c r="C10" s="75">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4767,7 +4759,7 @@
         <v>375</v>
       </c>
       <c r="C11" s="75">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4778,7 +4770,7 @@
         <v>376</v>
       </c>
       <c r="C12" s="76">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -4789,7 +4781,7 @@
         <v>378</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>437</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4800,7 +4792,7 @@
         <v>377</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>438</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4811,7 +4803,7 @@
         <v>379</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4822,7 +4814,7 @@
         <v>380</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>
@@ -4888,7 +4880,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
       <c r="C2" s="47" t="s">
         <v>263</v>
@@ -4907,7 +4899,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="C3" s="45" t="s">
         <v>262</v>
@@ -4933,7 +4925,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="C4" s="45" t="s">
         <v>262</v>
@@ -4950,7 +4942,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="45" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="F5" s="45" t="s">
         <v>274</v>
@@ -5129,7 +5121,7 @@
       </c>
       <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 56 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 100 mm y con un máximo de 67.4 mm/día.</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -5147,7 +5139,7 @@
       </c>
       <c r="L23" s="52" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 56 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 100 mm y con un máximo de 67.4 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
@@ -5162,7 +5154,7 @@
       </c>
       <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 54 mm y con un máximo de 53 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 112 mm y con un máximo de 58 mm/día.</v>
       </c>
       <c r="G24" s="53"/>
       <c r="H24" s="53"/>
@@ -5180,7 +5172,7 @@
       </c>
       <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 54 mm y con un máximo de 53 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 112 mm y con un máximo de 58 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
@@ -5195,13 +5187,13 @@
       </c>
       <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 29 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 57 mm y con un máximo de 30 mm/día.</v>
       </c>
       <c r="G25" s="52"/>
       <c r="H25" s="52"/>
       <c r="I25" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D25,IF(SANTALUCIA!C16=$E$8,$I$8,IF(SANTALUCIA!C16=$E$9,$I$9,$I$10)),$J$8,E25,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía. </v>
       </c>
       <c r="J25" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(SANTALUCIA!C36&gt;SANTALUCIA!C12,I13, IF(SANTALUCIA!C36=SANTALUCIA!C12,I14, I15)))</f>
@@ -5213,7 +5205,7 @@
       </c>
       <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 29 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 57 mm y con un máximo de 30 mm/día. Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5232,11 +5224,11 @@
       </c>
       <c r="I26" s="64" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de ; está en descenso en las ciudades de Salto Fray Bentos.</v>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Salto; se mantiene constante en la ciudad de  Paysandú; está en descenso en la ciudad de  Fray Bentos.</v>
       </c>
       <c r="J26" s="78" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C28&gt;URUGUAY!C7, URUGUAY!C30&gt;URUGUAY!C12, URUGUAY!C32&gt;URUGUAY!C17, URUGUAY!C34&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C28=URUGUAY!C7, URUGUAY!C30=URUGUAY!C12, URUGUAY!C32=URUGUAY!C17, URUGUAY!C34=URUGUAY!C22),I14, I15)))</f>
-        <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se prevé que el nivel descienda en los próximos días. </v>
+        <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
       </c>
       <c r="K26" s="78" t="str">
         <f>IF(AND(URUGUAY!C9="-", URUGUAY!C14="-", URUGUAY!C19="-", URUGUAY!C24="-"),"",IF(OR(URUGUAY!C28&gt;URUGUAY!C9, URUGUAY!C30&gt;URUGUAY!C14, URUGUAY!C32&gt;URUGUAY!C19,URUGUAY!C34&gt;URUGUAY!C24),_xlfn.CONCAT(F18,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),")."),_xlfn.CONCAT(F19,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),", pero no se puede descartar en su totalidad.")))</f>
@@ -5260,17 +5252,17 @@
       </c>
       <c r="H27" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E8,_xlfn.CONCAT(" ",$E$26,),""),IF(URUGUAY!$C$16=Tablas!E8,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E8,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E8,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Bella Unión Paysandú</v>
+        <v xml:space="preserve"> Bella Unión Salto</v>
       </c>
       <c r="I27" s="65" t="str">
         <f>_xlfn.CONCAT(I8,IF(G27&gt;1,$J$9,$J$8),H27, IF(G27=4,".", ";"))</f>
-        <v xml:space="preserve"> está en ascenso en las ciudades de Bella Unión Paysandú;</v>
+        <v xml:space="preserve"> está en ascenso en las ciudades de Bella Unión Salto;</v>
       </c>
       <c r="J27" s="78"/>
       <c r="K27" s="78"/>
       <c r="L27" s="78"/>
     </row>
-    <row r="28" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:13" ht="33" x14ac:dyDescent="0.3">
       <c r="C28" s="51"/>
       <c r="D28" s="51"/>
       <c r="E28" s="51" t="s">
@@ -5279,21 +5271,21 @@
       <c r="F28" s="77"/>
       <c r="G28" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v/>
+        <v xml:space="preserve"> Paysandú</v>
       </c>
       <c r="I28" s="65" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en la ciudad de ;</v>
+        <v xml:space="preserve"> se mantiene constante en la ciudad de  Paysandú;</v>
       </c>
       <c r="J28" s="78"/>
       <c r="K28" s="78"/>
       <c r="L28" s="78"/>
     </row>
-    <row r="29" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
       <c r="E29" s="51" t="s">
@@ -5302,15 +5294,15 @@
       <c r="F29" s="77"/>
       <c r="G29" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto Fray Bentos</v>
+        <v xml:space="preserve"> Fray Bentos</v>
       </c>
       <c r="I29" s="65" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
-        <v xml:space="preserve"> está en descenso en las ciudades de Salto Fray Bentos.</v>
+        <v xml:space="preserve"> está en descenso en la ciudad de  Fray Bentos.</v>
       </c>
       <c r="J29" s="78"/>
       <c r="K29" s="78"/>

</xml_diff>

<commit_message>
UPDATE AUTOMATIC DOWNLOAD FOR THE FLOOD REPORT
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEB8EF4-0734-4B2F-9164-A01C45A177D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E09FD6-4388-4BD2-A908-915BE20CED99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="437">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -198,24 +198,12 @@
     <t>anterior dato en Durazno Puente Nuevo (1 hora)</t>
   </si>
   <si>
-    <t>Lluvia registrada últimas 24 horas</t>
-  </si>
-  <si>
-    <t>Lluvia registrada últimas 48 horas</t>
-  </si>
-  <si>
-    <t>Lluvia registrada últimas 72 horas</t>
-  </si>
-  <si>
     <t>Lluvia pronosticada próximas 24 horas</t>
   </si>
   <si>
     <t>Lluvia pronosticada próximas 72 horas</t>
   </si>
   <si>
-    <t>Lluvia pronosticada próximas 48 horas</t>
-  </si>
-  <si>
     <t>Pronostico hidrologico en Sarandí del Yí</t>
   </si>
   <si>
@@ -1239,9 +1227,6 @@
     <t xml:space="preserve"> -</t>
   </si>
   <si>
-    <t xml:space="preserve">Estar atentos a los pronósticos meteorológicos que realiza el INUMET y a los próximos eventos de lluvia que se registren en la cuenca. </t>
-  </si>
-  <si>
     <t>Menor a 4 metros</t>
   </si>
   <si>
@@ -1263,9 +1248,6 @@
     <t>Tomar acción en realizar evacuaciones debido a la posibilidad de generarse inundaciones que afecten viviendas, infraestructura sensible y equipamientos urbanos</t>
   </si>
   <si>
-    <t>6000 y 7700</t>
-  </si>
-  <si>
     <t>Entre 20 y 21 julio</t>
   </si>
   <si>
@@ -1281,9 +1263,6 @@
     <t>Entre 21 y 22 de julio</t>
   </si>
   <si>
-    <t xml:space="preserve">Se mantiene incrementos de nivel en ríos y arroyos que transitan en la zona noreste, litoral norte, centro y este del país. </t>
-  </si>
-  <si>
     <t>Entre 8.33 a 9.00 metros</t>
   </si>
   <si>
@@ -1323,18 +1302,6 @@
     <t>Se espera incrementos leves de nivel en el río San José los cuales estarian por debajo de la cota de seguridad</t>
   </si>
   <si>
-    <t>Entre 4.80 a 7.00 metros</t>
-  </si>
-  <si>
-    <t>Se mantiene en ascenso los niveles de los ríos Cuariem y Arapey debido a las precipitaciones registrada los días anteriores. De acuerdo a datos brindados por CTM-Salto Grande</t>
-  </si>
-  <si>
-    <t>163 y 487</t>
-  </si>
-  <si>
-    <t>265 y 872</t>
-  </si>
-  <si>
     <t>En los últimos días se han registrados incrementos de nivel y caudal en los ríos Tacuarembó, Yí y el tramo del río Negro aguas arriba de la represa Rincón del Bonete. En la represa Hid. Constitución, UTE reporta que la previsión de erogados a erogar estaria entre 265 y 872 m3/s, sin embargo la previsión de niveles en Mercedes se mantendria por debajo de los 3.5 metros.</t>
   </si>
   <si>
@@ -1342,6 +1309,51 @@
   </si>
   <si>
     <t>Estar preparados a inundaciones en los primeros equipamientos colectivos expuesto de la localidad por la crecida. No descartar aún la posibilidad de afectación a las primeras viviendas de uso permanete en la trama urbana.</t>
+  </si>
+  <si>
+    <t>Acumulado 3 días</t>
+  </si>
+  <si>
+    <t>Acumulado diario</t>
+  </si>
+  <si>
+    <t>Acumulado semanal</t>
+  </si>
+  <si>
+    <t>Lluvia pronosticada próximas Semana</t>
+  </si>
+  <si>
+    <t>15000 y 16000</t>
+  </si>
+  <si>
+    <t>289 y 561</t>
+  </si>
+  <si>
+    <t>906 y 1182</t>
+  </si>
+  <si>
+    <t>Entre 6.30 y 6.80 metros</t>
+  </si>
+  <si>
+    <t>Menor a 10.90 metros</t>
+  </si>
+  <si>
+    <t>31 de julio</t>
+  </si>
+  <si>
+    <t>Entre 5.10 y 5.50 metros</t>
+  </si>
+  <si>
+    <t>Entre 2.50 a 2.80 metros</t>
+  </si>
+  <si>
+    <t>Estar preparados ante la posibilidad de generarse inundaciones en zona de vivienda en Bella Unión</t>
+  </si>
+  <si>
+    <t>Durante las últimas horas se ha observado la llegada de la onda de crecida del río Uruguay a la represa de Salto Grande. En Bella Unión, el nivel del río continúa en ascenso y podría alcanzar entre 6.30 y 6.80 metros entre hoy y mañana, aproximándose a la cota de seguridad de la localidad (6.30 metros). Por su parte, la CTM-Salto Grande reportó que en la ciudad de Salto el río no superará los 10.90 metros en las próximas horas, por lo que se mantendrá por debajo de su límite de seguridad (11.40 metros). Finalmente, la CARU prevé un nivel máximo de 5.30 metros para Paysandú y un nivel pronósticado de 2.75 metros para Fray Bentos, ubicando a ambas ciudades por debajo de sus cotas de seguridad.</t>
+  </si>
+  <si>
+    <t>El nivel del río Uruguay se mantiene en aguas medias altas</t>
   </si>
 </sst>
 </file>
@@ -2199,96 +2211,96 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="34" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="39">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46223</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="41">
         <f ca="1">$C$3-1</f>
-        <v>46222</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B5" s="31" t="s">
         <v>30</v>
       </c>
       <c r="C5" s="40">
         <f ca="1">$C$3-2</f>
-        <v>46221</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>32</v>
       </c>
       <c r="C6" s="41">
         <f ca="1">$C$3+1</f>
-        <v>46224</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>33</v>
       </c>
       <c r="C7" s="42">
         <f ca="1">$C$3+2</f>
-        <v>46225</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="40">
         <f ca="1">$C$3+3</f>
-        <v>46226</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>412</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>
@@ -2309,16 +2321,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B1" s="57" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C1" s="60" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="D1" s="60" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2326,13 +2338,13 @@
         <v>45224</v>
       </c>
       <c r="B2" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C2" s="61" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="D2" s="61" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2340,10 +2352,10 @@
         <v>45224</v>
       </c>
       <c r="B3" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C3" s="61" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2351,13 +2363,13 @@
         <v>45224</v>
       </c>
       <c r="B4" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2365,10 +2377,10 @@
         <v>45224</v>
       </c>
       <c r="B5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C5" s="61" t="s">
         <v>342</v>
-      </c>
-      <c r="C5" s="61" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2376,10 +2388,10 @@
         <v>45224</v>
       </c>
       <c r="B6" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D6" s="62" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2387,13 +2399,13 @@
         <v>45224</v>
       </c>
       <c r="B7" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C7" s="61" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="D7" s="61" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -2426,13 +2438,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="72">
-        <v>7.08</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2443,7 +2455,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="71">
-        <v>7.17</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2453,9 +2465,9 @@
       <c r="B4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="30" t="str">
+      <c r="C4" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2467,7 +2479,7 @@
       </c>
       <c r="C5" s="37" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2478,7 +2490,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="72">
-        <v>6.64</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2489,18 +2501,18 @@
         <v>7</v>
       </c>
       <c r="C7" s="71">
-        <v>6.48</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2510,9 +2522,9 @@
       <c r="B9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="30">
+      <c r="C9" s="30" t="str">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v>16</v>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2524,7 +2536,7 @@
       </c>
       <c r="C10" s="37" t="str">
         <f>IF(C9=0,"Permanece",IF(C9="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2535,7 +2547,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="72">
-        <v>5.49</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2546,15 +2558,15 @@
         <v>11</v>
       </c>
       <c r="C12" s="71">
-        <v>5.35</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C13" s="6"/>
     </row>
@@ -2567,7 +2579,7 @@
       </c>
       <c r="C14" s="30">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2579,7 +2591,7 @@
       </c>
       <c r="C15" s="37" t="str">
         <f>IF(C14=0,"Permanece",IF(C14="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2590,7 +2602,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="71">
-        <v>6.19</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2601,15 +2613,15 @@
         <v>14</v>
       </c>
       <c r="C17" s="71">
-        <v>6.03</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="C18" s="6"/>
     </row>
@@ -2622,7 +2634,7 @@
       </c>
       <c r="C19" s="30">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2634,183 +2646,183 @@
       </c>
       <c r="C20" s="37" t="str">
         <f>IF(C19=0,"Permanece",IF(C19="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
-        <v>51</v>
+        <v>423</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="74">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
-        <v>52</v>
+        <v>422</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="75">
-        <v>67.400000000000006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>53</v>
+        <v>424</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="75">
-        <v>23.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="75">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C25" s="75">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27" t="s">
-        <v>55</v>
+        <v>425</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C26" s="76">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B28" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="27" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>36</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>37</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="26" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>29</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="27" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="264.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -2861,35 +2873,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C2" s="71">
-        <v>5.4</v>
+        <v>4.53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C3" s="71">
-        <v>5.0999999999999996</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2897,11 +2909,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="30">
+        <v>80</v>
+      </c>
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>30</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2909,44 +2921,44 @@
         <v>44</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C7" s="71">
-        <v>7.7</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C8" s="71">
-        <v>7.51</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2954,11 +2966,11 @@
         <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="30">
+        <v>86</v>
+      </c>
+      <c r="C10" s="30" t="str">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>19</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2966,44 +2978,44 @@
         <v>44</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C12" s="71">
-        <v>7.33</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C13" s="71">
-        <v>7.21</v>
+        <v>5.44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3011,11 +3023,11 @@
         <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3023,7 +3035,7 @@
         <v>44</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
@@ -3032,152 +3044,152 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>51</v>
+        <v>423</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C17" s="74">
-        <v>58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>52</v>
+        <v>422</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C18" s="75">
-        <v>54</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>53</v>
+        <v>424</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C19" s="75">
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C20" s="75">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C21" s="75">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27" t="s">
-        <v>55</v>
+        <v>425</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C22" s="76">
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="26" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C23" s="73"/>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C24" s="9"/>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="26" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3266,35 +3278,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C2" s="72">
-        <v>3.51</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C3" s="71">
-        <v>3.49</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3302,11 +3314,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>164</v>
-      </c>
-      <c r="C5" s="30">
+        <v>160</v>
+      </c>
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>2</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3314,40 +3326,44 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C7" s="72"/>
+        <v>118</v>
+      </c>
+      <c r="C7" s="72">
+        <v>0.19</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C8" s="71"/>
+        <v>119</v>
+      </c>
+      <c r="C8" s="71">
+        <v>0.19</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3355,7 +3371,7 @@
         <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
@@ -3367,7 +3383,7 @@
         <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
@@ -3376,32 +3392,32 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C12" s="72">
-        <v>1.34</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C13" s="71">
-        <v>1.33</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C14" s="6"/>
     </row>
@@ -3410,11 +3426,11 @@
         <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3422,37 +3438,37 @@
         <v>44</v>
       </c>
       <c r="B16" s="36" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C17" s="71"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C18" s="71"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C19" s="6"/>
     </row>
@@ -3461,7 +3477,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C20" s="30">
         <f>IFERROR(ROUND(ABS(C17-C18)*100,0),"-")</f>
@@ -3473,7 +3489,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="36" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C21" s="37" t="str">
         <f>IFERROR(IF(C20=0,"Permanece",IF(SIGN(C20)=1,"Sube","Baja")),"-")</f>
@@ -3482,222 +3498,222 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>51</v>
+        <v>423</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C22" s="74">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>52</v>
+        <v>422</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C23" s="75">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
-        <v>53</v>
+        <v>424</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C24" s="76">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C25" s="75">
-        <v>5</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C26" s="75">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="27" t="s">
-        <v>55</v>
+        <v>425</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C27" s="76">
-        <v>0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="26" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="27" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="27" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -3747,35 +3763,35 @@
     </row>
     <row r="2" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C2" s="72">
-        <v>0.47</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C3" s="72">
-        <v>0.47</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3783,7 +3799,7 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
@@ -3795,7 +3811,7 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
@@ -3804,112 +3820,112 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>51</v>
+        <v>423</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C7" s="74">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>52</v>
+        <v>422</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C8" s="75">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="27" t="s">
-        <v>53</v>
+        <v>424</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C9" s="76">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C10" s="75">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C11" s="75">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>55</v>
+        <v>425</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C12" s="76">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="25" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -3960,35 +3976,35 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C2" s="72">
-        <v>4.58</v>
+        <v>8.5500000000000007</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C3" s="71">
-        <v>4.5999999999999996</v>
+        <v>8.52</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3996,11 +4012,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>207</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>203</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="D5" s="55"/>
     </row>
@@ -4009,44 +4025,44 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C7" s="72">
-        <v>4.05</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C8" s="71">
-        <v>4.04</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -4054,7 +4070,7 @@
         <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
@@ -4067,7 +4083,7 @@
         <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
@@ -4076,35 +4092,35 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C12" s="72">
-        <v>6.61</v>
+        <v>10.52</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C13" s="71">
-        <v>6.48</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -4112,7 +4128,7 @@
         <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
@@ -4124,7 +4140,7 @@
         <v>44</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
@@ -4133,35 +4149,35 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C17" s="72">
-        <v>3.01</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C18" s="71">
-        <v>3.01</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -4169,7 +4185,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C20" s="30">
         <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
@@ -4181,7 +4197,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="36" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
@@ -4190,35 +4206,35 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C22" s="72">
-        <v>2.42</v>
+        <v>2.2799999999999998</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C23" s="71">
-        <v>2.44</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -4226,7 +4242,7 @@
         <v>43</v>
       </c>
       <c r="B25" s="29" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C25" s="30" t="str">
         <f>IF((C22-C23)&gt;=0,ROUND((C22-C23)*100,0),"")</f>
@@ -4239,7 +4255,7 @@
         <v>44</v>
       </c>
       <c r="B26" s="36" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C26" s="37" t="str">
         <f>IF(C25=0,"Permanece",IF(C25="","Baja","Sube"))</f>
@@ -4249,121 +4265,123 @@
     </row>
     <row r="27" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>406</v>
+        <v>426</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>248</v>
+        <v>429</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>248</v>
+        <v>431</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="C31" s="10"/>
+        <v>194</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>431</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>248</v>
+        <v>432</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>248</v>
+        <v>431</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>248</v>
+        <v>433</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="264.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>398</v>
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -4413,35 +4431,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C2" s="72">
-        <v>7.17</v>
+        <v>8.9700000000000006</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C3" s="71">
-        <v>7.18</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4449,11 +4467,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>226</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>222</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4461,44 +4479,44 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C7" s="72">
-        <v>1.97</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C8" s="71">
-        <v>1.96</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4506,11 +4524,11 @@
         <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>232</v>
-      </c>
-      <c r="C10" s="30">
+        <v>228</v>
+      </c>
+      <c r="C10" s="30" t="str">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4518,91 +4536,91 @@
         <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C14" s="9"/>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="27" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C15" s="10"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C16" s="9"/>
     </row>
     <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="27" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C17" s="10"/>
     </row>
     <row r="18" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -4652,35 +4670,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="C2" s="72">
-        <v>4.5</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C3" s="71">
-        <v>4.3099999999999996</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4688,11 +4706,11 @@
         <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>369</v>
-      </c>
-      <c r="C5" s="30">
+        <v>365</v>
+      </c>
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>19</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4700,121 +4718,121 @@
         <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>51</v>
+        <v>423</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="C7" s="74">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>52</v>
+        <v>422</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C8" s="75">
-        <v>99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>53</v>
+        <v>424</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C9" s="75">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C10" s="75">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C11" s="75">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>55</v>
+        <v>425</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C12" s="76">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -4862,10 +4880,10 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="D1" s="49"/>
       <c r="E1" s="49"/>
@@ -4880,29 +4898,29 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="E2" s="47" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="F2" s="48" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G2" s="54"/>
       <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D3" s="45">
         <v>70</v>
@@ -4911,24 +4929,24 @@
         <v>200</v>
       </c>
       <c r="F3" s="45" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="I3" s="45" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="J3" s="45" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="K3" s="45" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D4" s="45">
         <v>30</v>
@@ -4937,23 +4955,23 @@
         <v>100</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="45" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="F5" s="45" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E7" s="47" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="G7" s="46"/>
       <c r="H7" s="46"/>
@@ -4965,49 +4983,49 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E8" s="45" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="F8" s="45" t="s">
+        <v>294</v>
+      </c>
+      <c r="I8" s="45" t="s">
         <v>298</v>
       </c>
-      <c r="I8" s="45" t="s">
-        <v>302</v>
-      </c>
       <c r="J8" s="45" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E9" s="45" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E10" s="45" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="I10" s="45" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C12" s="47" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D12" s="47" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="G12" s="46"/>
       <c r="H12" s="46"/>
@@ -5019,43 +5037,43 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D13" s="45" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="F13" s="45" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="I13" s="45" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D14" s="45" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="I14" s="45" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D15" s="45" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="I15" s="45" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="47" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D17" s="47" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E17" s="47" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="F17" s="46" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="G17" s="46"/>
       <c r="H17" s="46"/>
@@ -5067,67 +5085,67 @@
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F18" s="45" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="I18" s="45" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F19" s="45" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="I19" s="45" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="50" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="E22" s="50" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="F22" s="50" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="G22" s="50"/>
       <c r="H22" s="50"/>
       <c r="I22" s="50" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="J22" s="50" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="K22" s="50" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="L22" s="69" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="23" spans="3:13" s="63" customFormat="1" ht="99" x14ac:dyDescent="0.25">
       <c r="C23" s="63" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E23" s="63" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 100 mm y con un máximo de 67.4 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 1 mm y con un máximo de 1 mm/día.</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
       <c r="I23" s="52" t="str">
         <f>_xlfn.CONCAT($F$8,D23,IF(YI!C15=$E$8,$I$8,IF(YI!C15=$E$9,$I$9,$I$10)),$J$8,E23,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno. </v>
       </c>
       <c r="J23" s="52" t="str">
         <f>_xlfn.CONCAT(F13,IF(YI!C31&gt;YI!C11,I13, IF(YI!C31=YI!C11,I14, I15)))</f>
@@ -5139,22 +5157,22 @@
       </c>
       <c r="L23" s="52" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 100 mm y con un máximo de 67.4 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 1 mm y con un máximo de 1 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
       <c r="C24" s="51" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 112 mm y con un máximo de 58 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 64 mm y con un máximo de 32 mm/día.</v>
       </c>
       <c r="G24" s="53"/>
       <c r="H24" s="53"/>
@@ -5172,28 +5190,28 @@
       </c>
       <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 112 mm y con un máximo de 58 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 64 mm y con un máximo de 32 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
       <c r="C25" s="51" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 57 mm y con un máximo de 30 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 4 mm y con un máximo de 2 mm/día.</v>
       </c>
       <c r="G25" s="52"/>
       <c r="H25" s="52"/>
       <c r="I25" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D25,IF(SANTALUCIA!C16=$E$8,$I$8,IF(SANTALUCIA!C16=$E$9,$I$9,$I$10)),$J$8,E25,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía. </v>
       </c>
       <c r="J25" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(SANTALUCIA!C36&gt;SANTALUCIA!C12,I13, IF(SANTALUCIA!C36=SANTALUCIA!C12,I14, I15)))</f>
@@ -5205,18 +5223,18 @@
       </c>
       <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 57 mm y con un máximo de 30 mm/día. Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 4 mm y con un máximo de 2 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="51" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F26" s="77" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!#REF!)&gt;$D$3,SUM(URUGUAY!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!#REF!)&gt;$D$4,SUM(URUGUAY!#REF!)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!#REF!),$J$3,MAX(URUGUAY!#REF!),$K$3)</f>
@@ -5243,7 +5261,7 @@
       <c r="C27" s="51"/>
       <c r="D27" s="51"/>
       <c r="E27" s="51" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="F27" s="77"/>
       <c r="G27" s="58">
@@ -5266,7 +5284,7 @@
       <c r="C28" s="51"/>
       <c r="D28" s="51"/>
       <c r="E28" s="51" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="F28" s="77"/>
       <c r="G28" s="58">
@@ -5289,7 +5307,7 @@
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
       <c r="E29" s="51" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F29" s="77"/>
       <c r="G29" s="58">
@@ -5310,13 +5328,13 @@
     </row>
     <row r="30" spans="3:13" ht="66" x14ac:dyDescent="0.3">
       <c r="C30" s="51" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D30" s="51" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E30" s="51" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F30" s="52" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!#REF!)&gt;$D$3,SUM(NEGRO!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!#REF!)&gt;$D$4,SUM(NEGRO!#REF!)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!#REF!),$J$3,MAX(NEGRO!#REF!),$K$3)</f>
@@ -5326,7 +5344,7 @@
       <c r="H30" s="52"/>
       <c r="I30" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D30,IF(NEGRO!C11=$E$8,$I$8,IF(NEGRO!C11=$E$9,$I$9,$I$10)),$J$8,E30,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en ascenso en la ciudad de Mercedes. </v>
+        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en descenso en la ciudad de Mercedes. </v>
       </c>
       <c r="J30" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(NEGRO!C16&gt;NEGRO!C7,I13, IF(NEGRO!C16=NEGRO!C7,I14, I15)))</f>

</xml_diff>

<commit_message>
update python version of the repos and include notebook for pondering members ESP
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27969001-1268-4AB0-8F89-EDC1940BAFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31ABBF62-9016-4C87-AA76-EA4C14BA94E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="435">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -1227,9 +1227,6 @@
     <t xml:space="preserve"> -</t>
   </si>
   <si>
-    <t>Menor a 3 metros</t>
-  </si>
-  <si>
     <t>Mantener la vigilancia y el monitoreo en niveles de ríos y arroyos. Infórmese por fuentes oficiales</t>
   </si>
   <si>
@@ -1290,24 +1287,6 @@
     <t>Se observa un incremento de nivel del río San José el cual tiene posibilidad de aproximarse a la cota de aviso (3,32 metros) en las próximas horas. Debido a las precipitaciones pronosticadas, no se descarta que el río permanezca crecido en los próximos días. La probabilidad de llegar a cota de seguridad (7.40 m) es baja pero se actualizará información si se tiene un cambio en las condiciones hidrológicas</t>
   </si>
   <si>
-    <t>Menor a 6.00 metros</t>
-  </si>
-  <si>
-    <t>20 de agosto</t>
-  </si>
-  <si>
-    <t>Entre 10.30 a 11.00 metros</t>
-  </si>
-  <si>
-    <t>Entre 5.50 a 5.8 metros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Durante las últimas horas se ha observado un incremento del río Uruguay en la ciudad de Paysandú. Los ríos Dayman y Queguay han generado un caudal adicional al tramo del río Uruguay comprendido entre Salto y Paysandú el cual se espera que este por debajo de la cota de seguridad (6.0 m) definido para la ciudad. CTM Salto Grande reporta en su informe diario que en la ciudad de Salto el nivel del río variará entre 11.00 a 10.30 metros en las proximas horas. </t>
-  </si>
-  <si>
-    <t>Estar atentos a los cursos de agua urbanos y que aportan al río Uruguay en los departamentos de Salto y Paysandú</t>
-  </si>
-  <si>
     <t>Entre 10.72 y 11.68 metros</t>
   </si>
   <si>
@@ -1329,22 +1308,48 @@
     <t>Estar atentos y preparados a la posibilidad de un segundo evento de precipitación que podrian mantener las zonas inundadas en los próximos dias</t>
   </si>
   <si>
-    <t>8200 y 9200</t>
-  </si>
-  <si>
-    <t>3400 y 3849</t>
-  </si>
-  <si>
-    <t>4783 y 4886</t>
-  </si>
-  <si>
-    <t>Persiste niveles altos en los ríos Yí y Cebollatí</t>
-  </si>
-  <si>
     <t xml:space="preserve">Durante las últimas horas se ha observado el descenso del nivel del río Yí en la ciudad de Durazno. Sin embargo, el nivel actual reportado por la UTE muestra que aun el nivel del río está por encima de la cota de seguridad. </t>
   </si>
   <si>
     <t xml:space="preserve">En las últimas horas se ha observado semi-estacionario el nivel del río Negro en Mercedes </t>
+  </si>
+  <si>
+    <t>18500 y 18000</t>
+  </si>
+  <si>
+    <t>1606 y 1065</t>
+  </si>
+  <si>
+    <t>1781 y 1280</t>
+  </si>
+  <si>
+    <t>El río Uruguay registra niveles estables en Bella Unión y Salto.</t>
+  </si>
+  <si>
+    <t>Alrededor de 6,90 m</t>
+  </si>
+  <si>
+    <t>Menor a 12,10 m</t>
+  </si>
+  <si>
+    <t>12 de octubre</t>
+  </si>
+  <si>
+    <t>Alrededor de 6,40 m</t>
+  </si>
+  <si>
+    <t>Se recomienda mantener las medidas de respuesta y el seguimiento de la evolución de los niveles del río Uruguay, principalmente en Bella
+Unión y Paysandú, donde se han superado las cotas de seguridad. Asimismo, se recomienda mantener la vigilancia ante posibles
+nuevos incrementos de los niveles durante los próximos días.</t>
+  </si>
+  <si>
+    <t>Menor a 3,50 metros</t>
+  </si>
+  <si>
+    <t>13-14 de octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durante las últimas horas se ha observado una tendencia estable del río Uruguay en el tramo Paso de los Libres (Argentina) y Bella Unión. Sin embargo, se espera para los próximos días un repunte del río Uruguay debido a las lluvias registradas en la parte alta de la cuenca. Para las próximas horas se espera que el Río Uruguay en Bella Unión se encuentre estable y por debajo de los 6,90 metros. En Salto, de acuerdo a la CTM de Salto Grande, se espera que el nivel del río sea menor a 12,10 metros. En Paysandú, se espera que el nivel del río se mantenga por debajo de los 6,40 metros.  En Fray Bentos se espera que el nivel del río se mantenga inferior de 3,50 metros para los próximos 2 a 3 días. </t>
   </si>
 </sst>
 </file>
@@ -2208,7 +2213,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="39">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2220,7 +2225,7 @@
       </c>
       <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46258</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2232,7 +2237,7 @@
       </c>
       <c r="C4" s="41">
         <f ca="1">$C$3-1</f>
-        <v>46257</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2244,7 +2249,7 @@
       </c>
       <c r="C5" s="40">
         <f ca="1">$C$3-2</f>
-        <v>46256</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2256,7 +2261,7 @@
       </c>
       <c r="C6" s="41">
         <f ca="1">$C$3+1</f>
-        <v>46259</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2268,7 +2273,7 @@
       </c>
       <c r="C7" s="42">
         <f ca="1">$C$3+2</f>
-        <v>46260</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2280,7 +2285,7 @@
       </c>
       <c r="C8" s="40">
         <f ca="1">$C$3+3</f>
-        <v>46261</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2291,7 +2296,7 @@
         <v>167</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -2435,7 +2440,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="72">
-        <v>2.61</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2446,7 +2451,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="71">
-        <v>2.64</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2481,7 +2486,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="72">
-        <v>8</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2492,7 +2497,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="71">
-        <v>8.0500000000000007</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2513,9 +2518,9 @@
       <c r="B9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="30" t="str">
+      <c r="C9" s="30">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2527,7 +2532,7 @@
       </c>
       <c r="C10" s="37" t="str">
         <f>IF(C9=0,"Permanece",IF(C9="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2538,7 +2543,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="72">
-        <v>8.81</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2549,7 +2554,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="71">
-        <v>8.83</v>
+        <v>4.5599999999999996</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2593,7 +2598,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="71">
-        <v>10.02</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2604,7 +2609,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="71">
-        <v>10.039999999999999</v>
+        <v>2.3199999999999998</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2642,7 +2647,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>20</v>
@@ -2653,7 +2658,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>21</v>
@@ -2664,13 +2669,13 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="75">
-        <v>104</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2692,18 +2697,18 @@
         <v>24</v>
       </c>
       <c r="C25" s="75">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C26" s="76">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2802,7 +2807,7 @@
         <v>39</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2813,7 +2818,7 @@
         <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -2870,7 +2875,7 @@
         <v>78</v>
       </c>
       <c r="C2" s="71">
-        <v>4.2699999999999996</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2881,7 +2886,7 @@
         <v>79</v>
       </c>
       <c r="C3" s="71">
-        <v>4.2699999999999996</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2902,9 +2907,9 @@
       <c r="B5" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2916,7 +2921,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2927,7 +2932,7 @@
         <v>84</v>
       </c>
       <c r="C7" s="71">
-        <v>2.19</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2938,7 +2943,7 @@
         <v>85</v>
       </c>
       <c r="C8" s="71">
-        <v>2.2000000000000002</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2984,7 +2989,7 @@
         <v>90</v>
       </c>
       <c r="C12" s="71">
-        <v>3.28</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2995,7 +3000,7 @@
         <v>91</v>
       </c>
       <c r="C13" s="71">
-        <v>3.3</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3035,7 +3040,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>70</v>
@@ -3046,24 +3051,24 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>71</v>
       </c>
       <c r="C18" s="75">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C19" s="75">
-        <v>83</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -3074,7 +3079,7 @@
         <v>73</v>
       </c>
       <c r="C20" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3085,18 +3090,18 @@
         <v>74</v>
       </c>
       <c r="C21" s="75">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>75</v>
       </c>
       <c r="C22" s="76">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3151,7 +3156,7 @@
         <v>94</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3162,7 +3167,7 @@
         <v>95</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3173,7 +3178,7 @@
         <v>76</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3184,7 +3189,7 @@
         <v>77</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3279,7 +3284,7 @@
         <v>158</v>
       </c>
       <c r="C2" s="72">
-        <v>2.29</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3290,7 +3295,7 @@
         <v>159</v>
       </c>
       <c r="C3" s="71">
-        <v>2.3199999999999998</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3336,7 +3341,7 @@
         <v>118</v>
       </c>
       <c r="C7" s="72">
-        <v>4.4800000000000004</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3347,7 +3352,7 @@
         <v>119</v>
       </c>
       <c r="C8" s="71">
-        <v>4.4800000000000004</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3368,9 +3373,9 @@
       <c r="B10" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="30" t="str">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3382,7 +3387,7 @@
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3393,7 +3398,7 @@
         <v>162</v>
       </c>
       <c r="C12" s="72">
-        <v>5.8</v>
+        <v>4.3499999999999996</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3404,7 +3409,7 @@
         <v>163</v>
       </c>
       <c r="C13" s="71">
-        <v>5.84</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3447,7 +3452,9 @@
       <c r="B17" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C17" s="71"/>
+      <c r="C17" s="71">
+        <v>2.96</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
@@ -3456,7 +3463,9 @@
       <c r="B18" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C18" s="71"/>
+      <c r="C18" s="71">
+        <v>2.98</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
@@ -3476,7 +3485,7 @@
       </c>
       <c r="C20" s="30">
         <f>IFERROR(ROUND(ABS(C17-C18)*100,0),"-")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3488,12 +3497,12 @@
       </c>
       <c r="C21" s="37" t="str">
         <f>IFERROR(IF(C20=0,"Permanece",IF(SIGN(C20)=1,"Sube","Baja")),"-")</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>108</v>
@@ -3504,24 +3513,24 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>109</v>
       </c>
       <c r="C23" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>110</v>
       </c>
       <c r="C24" s="76">
-        <v>53</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3532,7 +3541,7 @@
         <v>111</v>
       </c>
       <c r="C25" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3543,18 +3552,18 @@
         <v>112</v>
       </c>
       <c r="C26" s="75">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>113</v>
       </c>
       <c r="C27" s="76">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -3601,7 +3610,7 @@
         <v>122</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3612,7 +3621,7 @@
         <v>123</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -3645,7 +3654,7 @@
         <v>124</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3656,7 +3665,7 @@
         <v>125</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3685,7 +3694,7 @@
         <v>114</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3696,7 +3705,7 @@
         <v>115</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -3752,7 +3761,7 @@
         <v>150</v>
       </c>
       <c r="C2" s="72">
-        <v>1.98</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3763,7 +3772,7 @@
         <v>151</v>
       </c>
       <c r="C3" s="72">
-        <v>2.0099999999999998</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3803,7 +3812,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>385</v>
@@ -3814,24 +3823,24 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>386</v>
       </c>
       <c r="C8" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="27" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>387</v>
       </c>
       <c r="C9" s="76">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3842,7 +3851,7 @@
         <v>388</v>
       </c>
       <c r="C10" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3853,18 +3862,18 @@
         <v>389</v>
       </c>
       <c r="C11" s="75">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>390</v>
       </c>
       <c r="C12" s="76">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3875,7 +3884,7 @@
         <v>156</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3886,7 +3895,7 @@
         <v>157</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3897,7 +3906,7 @@
         <v>391</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3965,7 +3974,7 @@
         <v>201</v>
       </c>
       <c r="C2" s="72">
-        <v>5.13</v>
+        <v>9.1199999999999992</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3976,7 +3985,7 @@
         <v>202</v>
       </c>
       <c r="C3" s="71">
-        <v>5.15</v>
+        <v>9.1199999999999992</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3997,9 +4006,9 @@
       <c r="B5" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="30" t="str">
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" s="55"/>
     </row>
@@ -4012,7 +4021,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -4023,7 +4032,7 @@
         <v>205</v>
       </c>
       <c r="C7" s="72">
-        <v>4.41</v>
+        <v>6.74</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -4034,7 +4043,7 @@
         <v>206</v>
       </c>
       <c r="C8" s="71">
-        <v>4.41</v>
+        <v>6.74</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -4081,7 +4090,7 @@
         <v>172</v>
       </c>
       <c r="C12" s="72">
-        <v>8.08</v>
+        <v>11.84</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -4092,7 +4101,7 @@
         <v>173</v>
       </c>
       <c r="C13" s="71">
-        <v>8.11</v>
+        <v>11.84</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -4113,9 +4122,9 @@
       <c r="B15" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="C15" s="30" t="str">
+      <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4127,7 +4136,7 @@
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4138,7 +4147,7 @@
         <v>209</v>
       </c>
       <c r="C17" s="72">
-        <v>5.0999999999999996</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -4149,7 +4158,7 @@
         <v>210</v>
       </c>
       <c r="C18" s="71">
-        <v>5.12</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -4170,9 +4179,9 @@
       <c r="B20" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="C20" s="30" t="str">
+      <c r="C20" s="30">
         <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4184,7 +4193,7 @@
       </c>
       <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -4195,7 +4204,7 @@
         <v>213</v>
       </c>
       <c r="C22" s="72">
-        <v>2.96</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -4206,7 +4215,7 @@
         <v>214</v>
       </c>
       <c r="C23" s="71">
-        <v>2.96</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -4254,7 +4263,7 @@
         <v>170</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -4265,7 +4274,7 @@
         <v>168</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>415</v>
+        <v>427</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4276,7 +4285,7 @@
         <v>169</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -4287,7 +4296,7 @@
         <v>193</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>417</v>
+        <v>428</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4298,7 +4307,7 @@
         <v>194</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -4309,7 +4318,7 @@
         <v>195</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>418</v>
+        <v>430</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4320,7 +4329,7 @@
         <v>196</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -4331,7 +4340,7 @@
         <v>199</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>394</v>
+        <v>432</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4342,10 +4351,10 @@
         <v>200</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="182.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="248.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="26" t="s">
         <v>60</v>
       </c>
@@ -4353,10 +4362,10 @@
         <v>192</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="28" t="s">
         <v>61</v>
       </c>
@@ -4364,7 +4373,7 @@
         <v>217</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>420</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -4420,7 +4429,7 @@
         <v>220</v>
       </c>
       <c r="C2" s="72">
-        <v>12.06</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4431,7 +4440,7 @@
         <v>221</v>
       </c>
       <c r="C3" s="71">
-        <v>12.04</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4454,7 +4463,7 @@
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4466,7 +4475,7 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4477,7 +4486,7 @@
         <v>226</v>
       </c>
       <c r="C7" s="72">
-        <v>6.09</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4488,7 +4497,7 @@
         <v>227</v>
       </c>
       <c r="C8" s="71">
-        <v>6.08</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4534,7 +4543,7 @@
         <v>233</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4545,7 +4554,7 @@
         <v>232</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4556,7 +4565,7 @@
         <v>240</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4567,7 +4576,7 @@
         <v>241</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4578,7 +4587,7 @@
         <v>234</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4589,7 +4598,7 @@
         <v>235</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4600,7 +4609,7 @@
         <v>242</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4611,7 +4620,7 @@
         <v>243</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -4667,7 +4676,7 @@
         <v>362</v>
       </c>
       <c r="C2" s="72">
-        <v>6.16</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4678,7 +4687,7 @@
         <v>363</v>
       </c>
       <c r="C3" s="71">
-        <v>6.18</v>
+        <v>2.0499999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4699,9 +4708,9 @@
       <c r="B5" s="29" t="s">
         <v>365</v>
       </c>
-      <c r="C5" s="30" t="str">
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4713,12 +4722,12 @@
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>367</v>
@@ -4729,7 +4738,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>368</v>
@@ -4740,13 +4749,13 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>369</v>
       </c>
       <c r="C9" s="75">
-        <v>195</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4757,7 +4766,7 @@
         <v>370</v>
       </c>
       <c r="C10" s="75">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4768,18 +4777,18 @@
         <v>371</v>
       </c>
       <c r="C11" s="75">
-        <v>35</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>372</v>
       </c>
       <c r="C12" s="76">
-        <v>36</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -4790,7 +4799,7 @@
         <v>374</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4801,7 +4810,7 @@
         <v>373</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4812,7 +4821,7 @@
         <v>375</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>426</v>
+        <v>419</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4823,7 +4832,7 @@
         <v>376</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -4889,7 +4898,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C2" s="47" t="s">
         <v>259</v>
@@ -4908,7 +4917,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C3" s="45" t="s">
         <v>258</v>
@@ -4934,7 +4943,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C4" s="45" t="s">
         <v>258</v>
@@ -4951,7 +4960,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="45" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F5" s="45" t="s">
         <v>270</v>
@@ -5130,7 +5139,7 @@
       </c>
       <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 104 mm y con un máximo de 104 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 49 mm/día.</v>
       </c>
       <c r="G23" s="52"/>
       <c r="H23" s="52"/>
@@ -5148,7 +5157,7 @@
       </c>
       <c r="L23" s="52" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 104 mm y con un máximo de 104 mm/día. Actualmente, el nivel del río Yí está en descenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 49 mm y con un máximo de 49 mm/día. Actualmente, el nivel del río Yí está en descenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
@@ -5163,7 +5172,7 @@
       </c>
       <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 83 mm y con un máximo de 83 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 61 mm y con un máximo de 51 mm/día.</v>
       </c>
       <c r="G24" s="53"/>
       <c r="H24" s="53"/>
@@ -5181,7 +5190,7 @@
       </c>
       <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 83 mm y con un máximo de 83 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 61 mm y con un máximo de 51 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
@@ -5196,7 +5205,7 @@
       </c>
       <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 53 mm y con un máximo de 53 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 28 mm y con un máximo de 27 mm/día.</v>
       </c>
       <c r="G25" s="52"/>
       <c r="H25" s="52"/>
@@ -5214,7 +5223,7 @@
       </c>
       <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 53 mm y con un máximo de 53 mm/día. Actualmente, el nivel del río Santa Lucía está en descenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 28 mm y con un máximo de 27 mm/día. Actualmente, el nivel del río Santa Lucía está en descenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -5233,7 +5242,7 @@
       </c>
       <c r="I26" s="64" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en la ciudad de ; se mantiene constante en las ciudades de Bella Unión Fray Bentos; está en descenso en las ciudades de Salto Paysandú.</v>
+        <v>Actualmente, el nivel del río Uruguay se mantiene constante en las ciudades de Bella Unión, Salto, Paysandú y Fray Bentos.</v>
       </c>
       <c r="J26" s="78" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C28&gt;URUGUAY!C7, URUGUAY!C30&gt;URUGUAY!C12, URUGUAY!C32&gt;URUGUAY!C17, URUGUAY!C34&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C28=URUGUAY!C7, URUGUAY!C30=URUGUAY!C12, URUGUAY!C32=URUGUAY!C17, URUGUAY!C34=URUGUAY!C22),I14, I15)))</f>
@@ -5271,7 +5280,7 @@
       <c r="K27" s="78"/>
       <c r="L27" s="78"/>
     </row>
-    <row r="28" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:13" ht="49.5" x14ac:dyDescent="0.3">
       <c r="C28" s="51"/>
       <c r="D28" s="51"/>
       <c r="E28" s="51" t="s">
@@ -5280,21 +5289,21 @@
       <c r="F28" s="77"/>
       <c r="G28" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H28" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Bella Unión Fray Bentos</v>
+        <v xml:space="preserve"> Bella Unión Salto Paysandú Fray Bentos</v>
       </c>
       <c r="I28" s="65" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en las ciudades de Bella Unión Fray Bentos;</v>
+        <v xml:space="preserve"> se mantiene constante en las ciudades de Bella Unión Salto Paysandú Fray Bentos.</v>
       </c>
       <c r="J28" s="78"/>
       <c r="K28" s="78"/>
       <c r="L28" s="78"/>
     </row>
-    <row r="29" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
       <c r="E29" s="51" t="s">
@@ -5303,15 +5312,15 @@
       <c r="F29" s="77"/>
       <c r="G29" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H29" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto Paysandú</v>
+        <v/>
       </c>
       <c r="I29" s="65" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
-        <v xml:space="preserve"> está en descenso en las ciudades de Salto Paysandú.</v>
+        <v xml:space="preserve"> está en descenso en la ciudad de .</v>
       </c>
       <c r="J29" s="78"/>
       <c r="K29" s="78"/>

</xml_diff>